<commit_message>
Record approved v5 boss parties, compatibility checks and next work
</commit_message>
<xml_diff>
--- a/docs/boss-party-review.xlsx
+++ b/docs/boss-party-review.xlsx
@@ -164,9 +164,9 @@
     <tableColumn id="4" name="원작 기준"/>
     <tableColumn id="5" name="원작 파티"/>
     <tableColumn id="6" name="고정 대표"/>
-    <tableColumn id="7" name="게임 검토안"/>
+    <tableColumn id="7" name="승인 적용 파티"/>
     <tableColumn id="8" name="원작 외 보충"/>
-    <tableColumn id="9" name="현재 게임 파티"/>
+    <tableColumn id="9" name="적용 전 파티"/>
     <tableColumn id="10" name="주의사항"/>
     <tableColumn id="11" name="출처"/>
     <tableColumn id="12" name="엑셀 행"/>
@@ -514,7 +514,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>게임 검토안</t>
+          <t>승인 적용 파티</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>현재 게임 파티</t>
+          <t>적용 전 파티</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>컨펌 대기 / 게임 미적용 / EXE 미생성</t>
+          <t>사용자 승인 / 새 원정 v5 적용 / EXE 미생성</t>
         </is>
       </c>
     </row>

</xml_diff>